<commit_message>
Update floor plan and booth assignments with SledLab
</commit_message>
<xml_diff>
--- a/docs/floorplan-2026/2026-vendor-assignments-sorted.xlsx
+++ b/docs/floorplan-2026/2026-vendor-assignments-sorted.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Booth Assignments" sheetId="1" r:id="R4ef755436f5340fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Booth Assignments" sheetId="1" r:id="R6a27589bbf134845"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -45,7 +45,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -65,6 +65,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF5F7F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -89,7 +94,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="21">
+  <x:cellXfs count="28">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -147,6 +152,23 @@
       <x:alignment horizontal="right" vertical="center" wrapText="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
@@ -157,8 +179,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BoothAssignmentsTable" displayName="BoothAssignmentsTable" ref="A5:B87" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:B87"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BoothAssignmentsTable" displayName="BoothAssignmentsTable" ref="A5:B88" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:B88"/>
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Booth"/>
     <x:tableColumn id="2" name="Company"/>
@@ -381,7 +403,7 @@
     </x:row>
     <x:row r="3" ht="20" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>Source: 2026 Colorado SnoMo Expo Vendor List.xlsx</x:v>
+        <x:v>Source: 2026 vendor list; organizer update October 18, 2026</x:v>
       </x:c>
       <x:c r="B3" s="5"/>
     </x:row>
@@ -1026,7 +1048,7 @@
         <x:v>327</x:v>
       </x:c>
       <x:c r="B84" s="18" t="str">
-        <x:v>TruckBoss</x:v>
+        <x:v>SledLab</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="20" customHeight="1">
@@ -1034,7 +1056,7 @@
         <x:v>328</x:v>
       </x:c>
       <x:c r="B85" s="20" t="str">
-        <x:v>Octane Addictions</x:v>
+        <x:v>TruckBoss</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="20" customHeight="1">
@@ -1053,10 +1075,18 @@
         <x:v>TFT-Sno Trac, LLC</x:v>
       </x:c>
     </x:row>
+    <x:row r="88" ht="20" customHeight="1">
+      <x:c r="A88" s="26" t="n">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="B88" s="27" t="str">
+        <x:v>Octane Addictions</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddc1c220a6554738"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9115df761d0946df"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>